<commit_message>
Update P2H Genset web improvements
</commit_message>
<xml_diff>
--- a/docs/Template-Impor-Akun.xlsx
+++ b/docs/Template-Impor-Akun.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
   <si>
     <t>No SID</t>
   </si>
@@ -50,7 +50,7 @@
     <t>Isi lembar "Akun"</t>
   </si>
   <si>
-    <t>Satu orang satu baris. Kolom yang wajib: No SID dan Nama. Teknisi dan pengawas juga WAJIB diisi Site-nya (mereka hanya akan melihat data di site itu). Peran kosong dianggap "teknisi".</t>
+    <t>Satu orang satu baris. Kolom yang wajib: No SID dan Nama. Semua peran selain admin WAJIB diisi Site-nya (mereka hanya akan melihat data di site itu). Peran kosong dianggap "teknisi".</t>
   </si>
   <si>
     <t>2</t>
@@ -119,6 +119,15 @@
     <t>Foreman / supervisor</t>
   </si>
   <si>
+    <t>teknisi &amp; pengawas</t>
+  </si>
+  <si>
+    <t>Gabungan dua peran: mengisi P2H dan juga memverifikasi P2H orang lain di site-nya. P2H yang ia isi sendiri tidak bisa ia verifikasi sendiri. Juga boleh ditulis: teknisi dan pengawas, teknisi/pengawas.</t>
+  </si>
+  <si>
+    <t>Orang yang merangkap teknisi dan pengawas</t>
+  </si>
+  <si>
     <t>admin</t>
   </si>
   <si>
@@ -131,7 +140,7 @@
     <t>Isi kolom "Site"</t>
   </si>
   <si>
-    <t>Binungan, Suaran, Gurimbang, Lati, Sambarata. WAJIB untuk teknisi dan pengawas: mereka hanya melihat dan mengisi genset di site itu. Kosongkan hanya untuk admin (admin melihat semua site).</t>
+    <t>Binungan, Suaran, Gurimbang, Lati, Sambarata. WAJIB untuk semua peran selain admin: mereka hanya melihat dan mengisi genset di site itu. Kosongkan hanya untuk admin (admin melihat semua site).</t>
   </si>
   <si>
     <t>Aturan penting</t>
@@ -146,7 +155,7 @@
     <t>Perusahaan dan Jabatan dicetak di PDF / Word / Excel (bagian tanda tangan), jadi tulis dengan benar.</t>
   </si>
   <si>
-    <t>Password awal: kalau dikosongkan, aplikasi membuatkan 8 huruf/angka acak. Kalau diisi sendiri, minimal 6 karakter. Apa pun pilihannya, orangnya wajib menggantinya saat masuk pertama.</t>
+    <t>Password awal: kalau dikosongkan, aplikasi membuatkan 8 huruf/angka acak. Kalau diisi sendiri, minimal 5 karakter. Apa pun pilihannya, orangnya wajib menggantinya saat masuk pertama.</t>
   </si>
   <si>
     <t>Sekali impor maksimal 500 baris. Baris yang gagal TIDAK dibuat dan alasannya ditampilkan; perbaiki lalu tempel ulang hanya baris yang gagal.</t>
@@ -186,6 +195,15 @@
   </si>
   <si>
     <t>PT Berau Coal · Admin aplikasi · admin · (kosong)</t>
+  </si>
+  <si>
+    <t>12348</t>
+  </si>
+  <si>
+    <t>Dewi</t>
+  </si>
+  <si>
+    <t>PT Mutiara Tanjung Lestari · Electrician · teknisi &amp; pengawas · Lati</t>
   </si>
 </sst>
 </file>
@@ -698,8 +716,7 @@
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="4" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
   </cols>
@@ -5229,10 +5246,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Peran" prompt="teknisi / pengawas / admin" showErrorMessage="1" errorStyle="warning" errorTitle="Peran" error="Pilih: teknisi, pengawas, atau admin." sqref="E2:E501">
-      <formula1>"teknisi,pengawas,admin"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Peran" prompt="teknisi / pengawas / teknisi &amp; pengawas / admin" showErrorMessage="1" errorStyle="warning" errorTitle="Peran" error="Pilih: teknisi, pengawas, teknisi &amp; pengawas, atau admin." sqref="E2:E501">
+      <formula1>"teknisi,pengawas,teknisi &amp; pengawas,admin"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Site" prompt="Binungan / Suaran / Gurimbang / Lati / Sambarata (wajib untuk teknisi dan pengawas)" showErrorMessage="1" errorStyle="warning" errorTitle="Site" error="Pilih salah satu site. Wajib untuk teknisi dan pengawas; kosongkan hanya untuk admin." sqref="F2:F501">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Site" prompt="Binungan / Suaran / Gurimbang / Lati / Sambarata (wajib selain admin)" showErrorMessage="1" errorStyle="warning" errorTitle="Site" error="Pilih salah satu site. Wajib selain admin; kosongkan hanya untuk admin." sqref="F2:F501">
       <formula1>"Binungan,Suaran,Gurimbang,Lati,Sambarata"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5246,7 +5263,7 @@
     <tabColor rgb="FF10130D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -5373,99 +5390,99 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B15" s="9" t="s">
+    <row r="14" ht="32" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="16" ht="48" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="8" t="s">
+      <c r="C14" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
+      <c r="D14" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" ht="46" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="8" t="s">
+    </row>
+    <row r="17" ht="48" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="9" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="20" ht="46" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
     </row>
     <row r="21" ht="46" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
     </row>
     <row r="22" ht="46" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" ht="46" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
+    <row r="24" ht="46" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C27" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D26" s="14" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="14" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5489,6 +5506,28 @@
       </c>
       <c r="D29" s="15" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -5500,13 +5539,13 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B17:D17"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B26:D26"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>